<commit_message>
Updating results iter 2 file
</commit_message>
<xml_diff>
--- a/data/results_iter2.xlsx
+++ b/data/results_iter2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danemerson/Documents/CMU/01_Research/Projects/CPA/Bayesian Optimization/cpa-bayesian-opt/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98645DE7-A8E1-2C41-8225-704CA7F097CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1857A16C-EECD-4A49-B0E1-AF8D189A538F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="19980" xr2:uid="{732449FA-1918-F249-870A-9891F3ECE17F}"/>
   </bookViews>
@@ -197,10 +197,10 @@
     <t>n=1 (5.5)</t>
   </si>
   <si>
-    <t xml:space="preserve">SD </t>
-  </si>
-  <si>
     <t>Experimental average</t>
+  </si>
+  <si>
+    <t>SD</t>
   </si>
 </sst>
 </file>
@@ -638,10 +638,10 @@
         <v>51</v>
       </c>
       <c r="O1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" t="s">
         <v>54</v>
-      </c>
-      <c r="P1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">

</xml_diff>